<commit_message>
added CU / RAMs tables
</commit_message>
<xml_diff>
--- a/compendium_schema (Joe).xlsx
+++ b/compendium_schema (Joe).xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ennsj\Documents\3. Management Domains\Interactive Tool\R Code\database_trial_jde\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ennsj\Documents\3. Management Domains\Interactive Tool\R Code\salmon_management_domains_compendium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7349C2E-122A-43B3-970E-6B23A54A7369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E36DB7-21E1-4F3F-B506-4304696FE263}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C8DE9B6A-1A32-438B-AB2C-1ED60489CD7B}"/>
+    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C8DE9B6A-1A32-438B-AB2C-1ED60489CD7B}"/>
   </bookViews>
   <sheets>
     <sheet name="Schema" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="64">
   <si>
     <t>Section</t>
   </si>
@@ -244,6 +244,12 @@
   </si>
   <si>
     <t>b any other fishery the minister of fisheries and oceans ministre</t>
+  </si>
+  <si>
+    <t>CU</t>
+  </si>
+  <si>
+    <t>RAMS</t>
   </si>
 </sst>
 </file>
@@ -428,16 +434,6 @@
     </dxf>
     <dxf>
       <font>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <b/>
         <i val="0"/>
         <strike val="0"/>
@@ -452,6 +448,16 @@
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <i val="0"/>
       </font>
     </dxf>
     <dxf>
@@ -491,7 +497,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4152C73F-C1A8-4E26-90FE-68AEE2561A7A}" name="Table1" displayName="Table1" ref="A1:A6" totalsRowShown="0" headerRowDxfId="9" dataDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4152C73F-C1A8-4E26-90FE-68AEE2561A7A}" name="Table1" displayName="Table1" ref="A1:A6" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
   <autoFilter ref="A1:A6" xr:uid="{4152C73F-C1A8-4E26-90FE-68AEE2561A7A}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{C9A0CD9E-9917-4190-8253-B4695A8A1E02}" name="legislation_table" dataDxfId="7"/>
@@ -501,6 +507,30 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{EB7250C4-9765-42FA-BDCB-69E1EDA90C21}" name="Table8" displayName="Table8" ref="I8:I9" totalsRowShown="0">
+  <autoFilter ref="I8:I9" xr:uid="{EB7250C4-9765-42FA-BDCB-69E1EDA90C21}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{2576247A-3067-4CAE-B18B-E28518257AB5}" name="RAMS"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{3163B7BB-0181-460C-9D7A-B1E529F4F148}" name="Table12" displayName="Table12" ref="A1:E6" totalsRowShown="0">
+  <autoFilter ref="A1:E6" xr:uid="{3163B7BB-0181-460C-9D7A-B1E529F4F148}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{97E988BA-A9A2-4B60-BB56-006542214541}" name="legislation_id"/>
+    <tableColumn id="2" xr3:uid="{1ECC0481-B447-4BA4-B6C9-4DE600E53D05}" name="jurisdiction"/>
+    <tableColumn id="3" xr3:uid="{FCFDDC17-3A30-471C-82AE-3F39F0C6F2DD}" name="legislation_type"/>
+    <tableColumn id="4" xr3:uid="{ACA07936-62C1-440F-9F67-871216C8E6B3}" name="act_name"/>
+    <tableColumn id="5" xr3:uid="{50473ABF-2B52-4B8D-B50E-FDD626C78053}" name="legislation_name"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{3E47224C-2C65-4BDB-B8EF-8C5455D97497}" name="Table13" displayName="Table13" ref="E1:I6" totalsRowShown="0">
   <autoFilter ref="E1:I6" xr:uid="{3E47224C-2C65-4BDB-B8EF-8C5455D97497}"/>
   <tableColumns count="5">
@@ -514,7 +544,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{ACE509D7-6417-4026-8DE6-1456837E4F15}" name="Table14" displayName="Table14" ref="A1:I6" totalsRowShown="0">
   <autoFilter ref="A1:I6" xr:uid="{ACE509D7-6417-4026-8DE6-1456837E4F15}"/>
   <tableColumns count="9">
@@ -533,10 +563,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D3628C70-7904-4F3A-AA07-E65176A44B4A}" name="Table2" displayName="Table2" ref="C1:C6" totalsRowShown="0" headerRowDxfId="8" dataDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D3628C70-7904-4F3A-AA07-E65176A44B4A}" name="Table2" displayName="Table2" ref="C1:C6" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
   <autoFilter ref="C1:C6" xr:uid="{D3628C70-7904-4F3A-AA07-E65176A44B4A}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{D73FCA12-B2A0-4DE1-9034-0E66AF885E4B}" name="provision_table" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{D73FCA12-B2A0-4DE1-9034-0E66AF885E4B}" name="provision_table" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -603,16 +633,12 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{3163B7BB-0181-460C-9D7A-B1E529F4F148}" name="Table12" displayName="Table12" ref="A1:E6" totalsRowShown="0">
-  <autoFilter ref="A1:E6" xr:uid="{3163B7BB-0181-460C-9D7A-B1E529F4F148}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{97E988BA-A9A2-4B60-BB56-006542214541}" name="legislation_id"/>
-    <tableColumn id="2" xr3:uid="{1ECC0481-B447-4BA4-B6C9-4DE600E53D05}" name="jurisdiction"/>
-    <tableColumn id="3" xr3:uid="{FCFDDC17-3A30-471C-82AE-3F39F0C6F2DD}" name="legislation_type"/>
-    <tableColumn id="4" xr3:uid="{ACA07936-62C1-440F-9F67-871216C8E6B3}" name="act_name"/>
-    <tableColumn id="5" xr3:uid="{50473ABF-2B52-4B8D-B50E-FDD626C78053}" name="legislation_name"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{85E6F4A1-3452-41DB-8DE6-81D124A04967}" name="Table7" displayName="Table7" ref="I1:I2" totalsRowShown="0">
+  <autoFilter ref="I1:I2" xr:uid="{85E6F4A1-3452-41DB-8DE6-81D124A04967}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{DA9F316B-35FB-4493-8E89-35918BA7F51C}" name="CU"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -913,7 +939,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9B93BC3-A7C7-4C7C-B60E-FF9A84A5B5E6}">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.36328125" customWidth="1"/>
@@ -921,11 +947,13 @@
     <col min="3" max="3" width="20.36328125" customWidth="1"/>
     <col min="4" max="4" width="4.36328125" customWidth="1"/>
     <col min="5" max="5" width="20.36328125" customWidth="1"/>
-    <col min="6" max="6" width="7.54296875" customWidth="1"/>
+    <col min="6" max="6" width="4.08984375" customWidth="1"/>
     <col min="7" max="7" width="32.81640625" customWidth="1"/>
+    <col min="8" max="8" width="3.54296875" customWidth="1"/>
+    <col min="9" max="9" width="31.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
@@ -938,8 +966,11 @@
       <c r="G1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="I1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>6</v>
       </c>
@@ -953,7 +984,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>7</v>
       </c>
@@ -967,7 +998,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>8</v>
       </c>
@@ -981,7 +1012,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
@@ -995,7 +1026,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>10</v>
       </c>
@@ -1006,7 +1037,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="E7" t="s">
         <v>13</v>
       </c>
@@ -1014,15 +1045,18 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="E8" s="7" t="s">
         <v>20</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="I8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="C9" s="2"/>
       <c r="E9" s="7" t="s">
         <v>22</v>
@@ -1032,33 +1066,33 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="E10" s="7" t="s">
         <v>16</v>
       </c>
       <c r="F10" s="7"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G11" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G12" s="10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G13" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G15" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G16" s="9" t="s">
         <v>17</v>
       </c>
@@ -1093,7 +1127,7 @@
   <headerFooter>
     <oddHeader>&amp;R&amp;"Calibri"&amp;12&amp;K000000 Unclassified - Non-Classifié&amp;1#_x000D_</oddHeader>
   </headerFooter>
-  <tableParts count="8">
+  <tableParts count="10">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
@@ -1102,6 +1136,8 @@
     <tablePart r:id="rId6"/>
     <tablePart r:id="rId7"/>
     <tablePart r:id="rId8"/>
+    <tablePart r:id="rId9"/>
+    <tablePart r:id="rId10"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Added datatables to schema
</commit_message>
<xml_diff>
--- a/compendium_schema (Joe).xlsx
+++ b/compendium_schema (Joe).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ennsj\Documents\3. Management Domains\Interactive Tool\R Code\salmon_management_domains_compendium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E36DB7-21E1-4F3F-B506-4304696FE263}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE77A96D-3051-4152-B3B2-4921D0E0581F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C8DE9B6A-1A32-438B-AB2C-1ED60489CD7B}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="65">
   <si>
     <t>Section</t>
   </si>
@@ -250,6 +250,9 @@
   </si>
   <si>
     <t>RAMS</t>
+  </si>
+  <si>
+    <t>Agencies</t>
   </si>
 </sst>
 </file>
@@ -517,6 +520,16 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9C4DBBFE-4A86-48E2-B101-152A6BF9BE52}" name="Table9" displayName="Table9" ref="I12:I13" totalsRowShown="0">
+  <autoFilter ref="I12:I13" xr:uid="{9C4DBBFE-4A86-48E2-B101-152A6BF9BE52}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{3566C0DB-5E9E-42CE-BE4F-C85C2DE094EA}" name="Agencies"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{3163B7BB-0181-460C-9D7A-B1E529F4F148}" name="Table12" displayName="Table12" ref="A1:E6" totalsRowShown="0">
   <autoFilter ref="A1:E6" xr:uid="{3163B7BB-0181-460C-9D7A-B1E529F4F148}"/>
   <tableColumns count="5">
@@ -530,7 +543,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{3E47224C-2C65-4BDB-B8EF-8C5455D97497}" name="Table13" displayName="Table13" ref="E1:I6" totalsRowShown="0">
   <autoFilter ref="E1:I6" xr:uid="{3E47224C-2C65-4BDB-B8EF-8C5455D97497}"/>
   <tableColumns count="5">
@@ -544,7 +557,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{ACE509D7-6417-4026-8DE6-1456837E4F15}" name="Table14" displayName="Table14" ref="A1:I6" totalsRowShown="0">
   <autoFilter ref="A1:I6" xr:uid="{ACE509D7-6417-4026-8DE6-1456837E4F15}"/>
   <tableColumns count="9">
@@ -1081,6 +1094,9 @@
       <c r="G12" s="10" t="s">
         <v>21</v>
       </c>
+      <c r="I12" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G13" t="s">
@@ -1127,7 +1143,7 @@
   <headerFooter>
     <oddHeader>&amp;R&amp;"Calibri"&amp;12&amp;K000000 Unclassified - Non-Classifié&amp;1#_x000D_</oddHeader>
   </headerFooter>
-  <tableParts count="10">
+  <tableParts count="11">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
@@ -1138,6 +1154,7 @@
     <tablePart r:id="rId8"/>
     <tablePart r:id="rId9"/>
     <tablePart r:id="rId10"/>
+    <tablePart r:id="rId11"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Changed the schema slightly to simplify the paragraph_label_table adding a label_type column
</commit_message>
<xml_diff>
--- a/compendium_schema (Joe).xlsx
+++ b/compendium_schema (Joe).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ennsj\Documents\3. Management Domains\Interactive Tool\R Code\salmon_management_domains_compendium\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{775C6CF8-5D92-4970-AE1C-8F1F1E744EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09343A6A-E18D-470A-B93F-05C36145E34F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C8DE9B6A-1A32-438B-AB2C-1ED60489CD7B}"/>
+    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C8DE9B6A-1A32-438B-AB2C-1ED60489CD7B}"/>
   </bookViews>
   <sheets>
     <sheet name="Schema" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="67">
   <si>
     <t>Section</t>
   </si>
@@ -253,13 +253,19 @@
   </si>
   <si>
     <t>Agencies</t>
+  </si>
+  <si>
+    <t>label_type</t>
+  </si>
+  <si>
+    <t>paragraph_id</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -284,22 +290,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF0070C0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="0" tint="-0.34998626667073579"/>
       <name val="Calibri"/>
@@ -309,23 +299,13 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="5" tint="-0.249977111117893"/>
+      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFCC00CC"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -351,23 +331,203 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="18">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -427,16 +587,6 @@
     </dxf>
     <dxf>
       <font>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <b/>
         <i val="0"/>
         <strike val="0"/>
@@ -451,16 +601,6 @@
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <i val="0"/>
       </font>
     </dxf>
     <dxf>
@@ -500,18 +640,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4152C73F-C1A8-4E26-90FE-68AEE2561A7A}" name="Table1" displayName="Table1" ref="A1:A6" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4152C73F-C1A8-4E26-90FE-68AEE2561A7A}" name="Table1" displayName="Table1" ref="A1:A6" totalsRowShown="0" headerRowDxfId="17" dataDxfId="8">
   <autoFilter ref="A1:A6" xr:uid="{4152C73F-C1A8-4E26-90FE-68AEE2561A7A}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{C9A0CD9E-9917-4190-8253-B4695A8A1E02}" name="legislation_table" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{C9A0CD9E-9917-4190-8253-B4695A8A1E02}" name="legislation_table" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{EB7250C4-9765-42FA-BDCB-69E1EDA90C21}" name="Table8" displayName="Table8" ref="I8:I9" totalsRowShown="0">
-  <autoFilter ref="I8:I9" xr:uid="{EB7250C4-9765-42FA-BDCB-69E1EDA90C21}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{EB7250C4-9765-42FA-BDCB-69E1EDA90C21}" name="Table8" displayName="Table8" ref="K8:K9" totalsRowShown="0">
+  <autoFilter ref="K8:K9" xr:uid="{EB7250C4-9765-42FA-BDCB-69E1EDA90C21}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{2576247A-3067-4CAE-B18B-E28518257AB5}" name="RAMS"/>
   </tableColumns>
@@ -520,8 +660,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9C4DBBFE-4A86-48E2-B101-152A6BF9BE52}" name="Table9" displayName="Table9" ref="I12:I13" totalsRowShown="0">
-  <autoFilter ref="I12:I13" xr:uid="{9C4DBBFE-4A86-48E2-B101-152A6BF9BE52}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9C4DBBFE-4A86-48E2-B101-152A6BF9BE52}" name="Table9" displayName="Table9" ref="K12:K13" totalsRowShown="0">
+  <autoFilter ref="K12:K13" xr:uid="{9C4DBBFE-4A86-48E2-B101-152A6BF9BE52}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{3566C0DB-5E9E-42CE-BE4F-C85C2DE094EA}" name="Agencies"/>
   </tableColumns>
@@ -548,7 +688,7 @@
   <autoFilter ref="E1:I6" xr:uid="{3E47224C-2C65-4BDB-B8EF-8C5455D97497}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{183788B4-1C0A-451F-B755-7036D9C5E554}" name="legislation_id"/>
-    <tableColumn id="2" xr3:uid="{188CFBD6-492F-41FB-88A5-2D67A4C150AA}" name="Section" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{188CFBD6-492F-41FB-88A5-2D67A4C150AA}" name="Section" dataDxfId="15"/>
     <tableColumn id="3" xr3:uid="{51465D24-FE20-47A4-B83C-7018836C283D}" name="Heading"/>
     <tableColumn id="4" xr3:uid="{D7C77C11-08FA-4AFD-88D5-61DE05CD9927}" name="Paragraph"/>
     <tableColumn id="5" xr3:uid="{22417FF5-1875-43D6-93E8-D7ED01F1AFB0}" name="provision_id"/>
@@ -562,13 +702,13 @@
   <autoFilter ref="A1:I6" xr:uid="{ACE509D7-6417-4026-8DE6-1456837E4F15}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{306BDDCE-9716-46D7-BA5D-BC41DBFFF7A8}" name="provision_id"/>
-    <tableColumn id="2" xr3:uid="{A1B95BA9-0E8F-4A91-BC88-E752D44EFD36}" name="cleaned_paragraph" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{A1B95BA9-0E8F-4A91-BC88-E752D44EFD36}" name="cleaned_paragraph" dataDxfId="14"/>
     <tableColumn id="3" xr3:uid="{79B9AD73-8C25-4DF3-85E3-B217E02B834D}" name="scope"/>
     <tableColumn id="4" xr3:uid="{61BF9428-E7D0-47A7-AF3C-F7F654175CA3}" name="management_domain"/>
     <tableColumn id="5" xr3:uid="{9B350443-8771-43CE-810A-78E373E90914}" name="iucn_l2"/>
-    <tableColumn id="6" xr3:uid="{0D675FA4-3229-482B-A13F-CBC71BBE1AD1}" name="iucn_keyword" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{0D675FA4-3229-482B-A13F-CBC71BBE1AD1}" name="iucn_keyword" dataDxfId="13"/>
     <tableColumn id="7" xr3:uid="{FD586531-F72C-463D-A186-417D21F89CED}" name="clause_type"/>
-    <tableColumn id="8" xr3:uid="{16043E55-CD60-495C-8400-44BFB7262EFB}" name="clause_type_keyword" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{16043E55-CD60-495C-8400-44BFB7262EFB}" name="clause_type_keyword" dataDxfId="12"/>
     <tableColumn id="9" xr3:uid="{55DF37BB-8C8E-4884-B679-CD85F0D287B7}" name="label_id"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -576,58 +716,58 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D3628C70-7904-4F3A-AA07-E65176A44B4A}" name="Table2" displayName="Table2" ref="C1:C6" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D3628C70-7904-4F3A-AA07-E65176A44B4A}" name="Table2" displayName="Table2" ref="C1:C6" totalsRowShown="0" headerRowDxfId="16" dataDxfId="6">
   <autoFilter ref="C1:C6" xr:uid="{D3628C70-7904-4F3A-AA07-E65176A44B4A}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{D73FCA12-B2A0-4DE1-9034-0E66AF885E4B}" name="provision_table" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{D73FCA12-B2A0-4DE1-9034-0E66AF885E4B}" name="provision_table" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E67CBFAF-E2A1-44FD-A774-040B57044B3F}" name="Table3" displayName="Table3" ref="E1:E10" totalsRowShown="0">
-  <autoFilter ref="E1:E10" xr:uid="{E67CBFAF-E2A1-44FD-A774-040B57044B3F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E67CBFAF-E2A1-44FD-A774-040B57044B3F}" name="Table3" displayName="Table3" ref="E1:E5" totalsRowShown="0" dataDxfId="4">
+  <autoFilter ref="E1:E5" xr:uid="{E67CBFAF-E2A1-44FD-A774-040B57044B3F}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{6CDA10F9-AAA7-4235-9F54-34591AF6CB0F}" name="Provision Label Table"/>
+    <tableColumn id="1" xr3:uid="{6CDA10F9-AAA7-4235-9F54-34591AF6CB0F}" name="Provision Label Table" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D746B4DA-D1AC-47AB-8D62-85BEF5C48579}" name="Table4" displayName="Table4" ref="G1:G5" totalsRowShown="0">
-  <autoFilter ref="G1:G5" xr:uid="{D746B4DA-D1AC-47AB-8D62-85BEF5C48579}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D746B4DA-D1AC-47AB-8D62-85BEF5C48579}" name="Table4" displayName="Table4" ref="I1:I5" totalsRowShown="0" dataDxfId="10">
+  <autoFilter ref="I1:I5" xr:uid="{D746B4DA-D1AC-47AB-8D62-85BEF5C48579}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{C323B4AC-78BB-49C5-8584-55C8E5EE63E5}" name="management_domain_threat_table"/>
+    <tableColumn id="1" xr3:uid="{C323B4AC-78BB-49C5-8584-55C8E5EE63E5}" name="management_domain_threat_table" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{61695DF6-56F0-4ED1-A0E9-E48FE8873BD0}" name="Table5" displayName="Table5" ref="G7:G9" totalsRowShown="0">
-  <autoFilter ref="G7:G9" xr:uid="{61695DF6-56F0-4ED1-A0E9-E48FE8873BD0}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{61695DF6-56F0-4ED1-A0E9-E48FE8873BD0}" name="Table5" displayName="Table5" ref="G1:G3" totalsRowShown="0" dataDxfId="2">
+  <autoFilter ref="G1:G3" xr:uid="{61695DF6-56F0-4ED1-A0E9-E48FE8873BD0}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{2FC4FDFA-CC28-45E6-AE77-40CEA81F47F6}" name="iucn_l2_keywords"/>
+    <tableColumn id="1" xr3:uid="{2FC4FDFA-CC28-45E6-AE77-40CEA81F47F6}" name="iucn_l2_keywords" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{E72814D5-4D64-44E7-AC71-E374B0326BA4}" name="Table6" displayName="Table6" ref="G11:G13" totalsRowShown="0">
-  <autoFilter ref="G11:G13" xr:uid="{E72814D5-4D64-44E7-AC71-E374B0326BA4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{E72814D5-4D64-44E7-AC71-E374B0326BA4}" name="Table6" displayName="Table6" ref="G5:G7" totalsRowShown="0" dataDxfId="0">
+  <autoFilter ref="G5:G7" xr:uid="{E72814D5-4D64-44E7-AC71-E374B0326BA4}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{538DF6E0-C1CB-4D72-B1C0-1DF9D9675B41}" name="clause_type_keywords"/>
+    <tableColumn id="1" xr3:uid="{538DF6E0-C1CB-4D72-B1C0-1DF9D9675B41}" name="clause_type_keywords" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{864CAB8D-D456-474C-82A8-DE202ED80D50}" name="Table10" displayName="Table10" ref="G15:G17" totalsRowShown="0">
-  <autoFilter ref="G15:G17" xr:uid="{864CAB8D-D456-474C-82A8-DE202ED80D50}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{864CAB8D-D456-474C-82A8-DE202ED80D50}" name="Table10" displayName="Table10" ref="G9:G11" totalsRowShown="0">
+  <autoFilter ref="G9:G11" xr:uid="{864CAB8D-D456-474C-82A8-DE202ED80D50}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{90189859-0AE6-45A2-9A02-9FEBB0E11F6E}" name="salmon_scope_keywords"/>
   </tableColumns>
@@ -636,8 +776,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AB6B0853-3F5B-432F-B49B-5BE462057A66}" name="Table11" displayName="Table11" ref="G19:G22" totalsRowShown="0">
-  <autoFilter ref="G19:G22" xr:uid="{AB6B0853-3F5B-432F-B49B-5BE462057A66}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AB6B0853-3F5B-432F-B49B-5BE462057A66}" name="Table11" displayName="Table11" ref="G13:G16" totalsRowShown="0">
+  <autoFilter ref="G13:G16" xr:uid="{AB6B0853-3F5B-432F-B49B-5BE462057A66}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{B2A5DDE4-1A05-41C6-BEDB-173D997F5D8E}" name="governance_keywords"/>
   </tableColumns>
@@ -646,8 +786,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{85E6F4A1-3452-41DB-8DE6-81D124A04967}" name="Table7" displayName="Table7" ref="I1:I2" totalsRowShown="0">
-  <autoFilter ref="I1:I2" xr:uid="{85E6F4A1-3452-41DB-8DE6-81D124A04967}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{85E6F4A1-3452-41DB-8DE6-81D124A04967}" name="Table7" displayName="Table7" ref="K1:K2" totalsRowShown="0">
+  <autoFilter ref="K1:K2" xr:uid="{85E6F4A1-3452-41DB-8DE6-81D124A04967}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{DA9F316B-35FB-4493-8E89-35918BA7F51C}" name="CU"/>
   </tableColumns>
@@ -952,7 +1092,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9B93BC3-A7C7-4C7C-B60E-FF9A84A5B5E6}">
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.36328125" customWidth="1"/>
@@ -962,11 +1102,13 @@
     <col min="5" max="5" width="20.36328125" customWidth="1"/>
     <col min="6" max="6" width="4.08984375" customWidth="1"/>
     <col min="7" max="7" width="32.81640625" customWidth="1"/>
-    <col min="8" max="8" width="3.54296875" customWidth="1"/>
-    <col min="9" max="9" width="31.26953125" customWidth="1"/>
+    <col min="8" max="8" width="5.26953125" customWidth="1"/>
+    <col min="9" max="9" width="32.81640625" customWidth="1"/>
+    <col min="10" max="10" width="3.54296875" customWidth="1"/>
+    <col min="11" max="11" width="31.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
@@ -977,166 +1119,165 @@
         <v>3</v>
       </c>
       <c r="G1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>6</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" t="s">
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E6" s="5"/>
+      <c r="G6" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G7" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="E8" s="4"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="K8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C9" s="2"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="K12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G13" t="s">
+        <v>29</v>
+      </c>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G14" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G5" s="9" t="s">
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G15" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="E7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="E8" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="I8" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C9" s="2"/>
-      <c r="E9" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F9" s="7"/>
-      <c r="G9" t="s">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G16" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="E10" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F10" s="7"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="G11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="G12" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="I12" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="G13" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="G15" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="G16" s="9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" spans="7:7" x14ac:dyDescent="0.35">
-      <c r="G17" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="19" spans="7:7" x14ac:dyDescent="0.35">
-      <c r="G19" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="20" spans="7:7" x14ac:dyDescent="0.35">
-      <c r="G20" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="21" spans="7:7" x14ac:dyDescent="0.35">
-      <c r="G21" s="9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22" spans="7:7" x14ac:dyDescent="0.35">
-      <c r="G22" t="s">
-        <v>26</v>
-      </c>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6"/>
+    </row>
+    <row r="21" spans="8:9" x14ac:dyDescent="0.35">
+      <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1416,9 +1557,9 @@
     <col min="2" max="2" width="20.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="47.08984375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.26953125" customWidth="1"/>
-    <col min="6" max="6" width="14.54296875" style="7" customWidth="1"/>
+    <col min="6" max="6" width="14.54296875" style="4" customWidth="1"/>
     <col min="7" max="7" width="12.7265625" customWidth="1"/>
-    <col min="8" max="8" width="21" style="7" customWidth="1"/>
+    <col min="8" max="8" width="21" style="4" customWidth="1"/>
     <col min="9" max="9" width="9.36328125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1426,7 +1567,7 @@
       <c r="A1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C1" t="s">
@@ -1438,13 +1579,13 @@
       <c r="E1" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="4" t="s">
         <v>20</v>
       </c>
       <c r="G1" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="4" t="s">
         <v>22</v>
       </c>
       <c r="I1" t="s">
@@ -1455,7 +1596,7 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="4" t="s">
         <v>47</v>
       </c>
       <c r="C2" t="s">
@@ -1467,13 +1608,13 @@
       <c r="E2" t="s">
         <v>50</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="4" t="s">
         <v>51</v>
       </c>
       <c r="G2" t="s">
         <v>52</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="4" t="s">
         <v>53</v>
       </c>
       <c r="I2">
@@ -1484,7 +1625,7 @@
       <c r="A3">
         <v>6</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="4" t="s">
         <v>54</v>
       </c>
       <c r="C3" t="s">
@@ -1496,13 +1637,13 @@
       <c r="E3" t="s">
         <v>50</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G3" t="s">
         <v>56</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="4" t="s">
         <v>57</v>
       </c>
       <c r="I3">
@@ -1513,7 +1654,7 @@
       <c r="A4">
         <v>6</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="4" t="s">
         <v>54</v>
       </c>
       <c r="C4" t="s">
@@ -1525,13 +1666,13 @@
       <c r="E4" t="s">
         <v>50</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="4" t="s">
         <v>58</v>
       </c>
       <c r="G4" t="s">
         <v>56</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="4" t="s">
         <v>57</v>
       </c>
       <c r="I4">
@@ -1542,7 +1683,7 @@
       <c r="A5">
         <v>7</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="4" t="s">
         <v>59</v>
       </c>
       <c r="C5" t="s">
@@ -1554,13 +1695,13 @@
       <c r="E5" t="s">
         <v>50</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G5" t="s">
         <v>60</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="4" t="s">
         <v>60</v>
       </c>
       <c r="I5">
@@ -1571,7 +1712,7 @@
       <c r="A6">
         <v>8</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="4" t="s">
         <v>61</v>
       </c>
       <c r="C6" t="s">
@@ -1583,13 +1724,13 @@
       <c r="E6" t="s">
         <v>50</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G6" t="s">
         <v>60</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="4" t="s">
         <v>60</v>
       </c>
       <c r="I6">

</xml_diff>